<commit_message>
committing before pulling most recent pest run
</commit_message>
<xml_diff>
--- a/data_prep/horizontal_K_from_Amod.xlsx
+++ b/data_prep/horizontal_K_from_Amod.xlsx
@@ -5,7 +5,7 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pestPrep\gsflow\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git_repos\alameda\pestPrep\data_prep\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="15">
   <si>
     <t>m/s</t>
   </si>
@@ -63,13 +63,19 @@
   </si>
   <si>
     <t>ft/s</t>
+  </si>
+  <si>
+    <t>ft/day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colluvium </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -94,14 +100,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
+      <sz val="12"/>
       <color rgb="FF222222"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -144,20 +143,27 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="11" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="11" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -507,248 +513,366 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="18.375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.375" customWidth="1"/>
-    <col min="5" max="5" width="13.625" customWidth="1"/>
-    <col min="6" max="6" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11" style="7"/>
+    <col min="2" max="2" width="18.375" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.375" style="7" customWidth="1"/>
+    <col min="4" max="4" width="11" style="7"/>
+    <col min="5" max="5" width="13.625" style="7" customWidth="1"/>
+    <col min="6" max="6" width="11.625" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="11" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="6" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:6" s="2" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="5">
         <v>0.01</v>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="5">
         <v>5.9999999999999995E-4</v>
       </c>
-      <c r="F2" s="8">
+      <c r="F2" s="6">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="5">
         <f>D2*3.28084</f>
         <v>3.2808400000000001E-2</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="5">
         <f>E2*3.28084</f>
         <v>1.9685039999999998E-3</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="5">
         <f>F2*3.28084</f>
         <v>6.56168</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
+    <row r="4" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="10">
+        <v>1</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="12">
+        <f>D3*86400</f>
+        <v>2834.6457600000003</v>
+      </c>
+      <c r="E4" s="12">
+        <f t="shared" ref="E4:F4" si="0">E3*86400</f>
+        <v>170.07874559999999</v>
+      </c>
+      <c r="F4" s="12">
+        <f t="shared" si="0"/>
+        <v>566929.152</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D5" s="5">
         <v>4.0000000000000002E-4</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E5" s="5">
         <v>4.0000000000000003E-5</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F5" s="5">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="7">
-        <f>D4*3.28084</f>
+      <c r="D6" s="5">
+        <f>D5*3.28084</f>
         <v>1.3123360000000001E-3</v>
       </c>
-      <c r="E5" s="3">
-        <f>E4*3.28084</f>
+      <c r="E6" s="5">
+        <f>E5*3.28084</f>
         <v>1.3123360000000001E-4</v>
       </c>
-      <c r="F5" s="7">
-        <f>F4*3.28084</f>
+      <c r="F6" s="5">
+        <f>F5*3.28084</f>
         <v>3.2808400000000001E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="4">
+    <row r="7" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="10">
+        <v>2</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="12">
+        <f>D6*86400</f>
+        <v>113.3858304</v>
+      </c>
+      <c r="E7" s="12">
+        <f t="shared" ref="E7:F7" si="1">E6*86400</f>
+        <v>11.338583040000001</v>
+      </c>
+      <c r="F7" s="12">
+        <f t="shared" si="1"/>
+        <v>283.46457600000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
         <v>3</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B8" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D8" s="5">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E8" s="5">
         <v>1E-4</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F8" s="5">
         <v>0.02</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A7" s="4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
         <v>3</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B9" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="7">
-        <f>D6*3.28084</f>
+      <c r="D9" s="5">
+        <f>D8*3.28084</f>
         <v>9.8425200000000004E-3</v>
       </c>
-      <c r="E7" s="3">
-        <f>E6*3.28084</f>
+      <c r="E9" s="5">
+        <f>E8*3.28084</f>
         <v>3.2808400000000003E-4</v>
       </c>
-      <c r="F7" s="7">
-        <f>F6*3.28084</f>
+      <c r="F9" s="5">
+        <f>F8*3.28084</f>
         <v>6.5616800000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="4">
+    <row r="10" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="14">
+        <v>3</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="12">
+        <f>D9*86400</f>
+        <v>850.39372800000001</v>
+      </c>
+      <c r="E10" s="12">
+        <f t="shared" ref="E10:F10" si="2">E9*86400</f>
+        <v>28.346457600000001</v>
+      </c>
+      <c r="F10" s="12">
+        <f t="shared" si="2"/>
+        <v>5669.2915200000007</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
         <v>4</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B11" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C11" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D11" s="9">
         <v>4.9999999999999998E-8</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E11" s="9">
         <v>5.0000000000000001E-9</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F11" s="9">
         <v>4.9999999999999998E-7</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A9" s="4">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="8">
         <v>4</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B12" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="3">
-        <f>D8*3.28084</f>
+      <c r="D12" s="9">
+        <f>D11*3.28084</f>
         <v>1.6404199999999998E-7</v>
       </c>
-      <c r="E9" s="3">
-        <f>E8*3.28084</f>
+      <c r="E12" s="9">
+        <f>E11*3.28084</f>
         <v>1.64042E-8</v>
       </c>
-      <c r="F9" s="3">
-        <f>F8*3.28084</f>
+      <c r="F12" s="9">
+        <f>F11*3.28084</f>
         <v>1.6404199999999999E-6</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A10" s="4">
+    <row r="13" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="14">
+        <v>4</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="12">
+        <f>D12*86400</f>
+        <v>1.4173228799999998E-2</v>
+      </c>
+      <c r="E13" s="12">
+        <f t="shared" ref="E13:F13" si="3">E12*86400</f>
+        <v>1.4173228800000001E-3</v>
+      </c>
+      <c r="F13" s="12">
+        <f t="shared" si="3"/>
+        <v>0.14173228799999998</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="8">
         <v>5</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B14" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C14" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D14" s="9">
         <v>4.9999999999999999E-13</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E14" s="4">
         <v>0</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F14" s="9">
         <v>5.0000000000000002E-11</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A11" s="4">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="8">
         <v>5</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B15" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C15" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="3">
-        <f t="shared" ref="D11:F11" si="0">D10*3.28084</f>
+      <c r="D15" s="9">
+        <f t="shared" ref="D15:F15" si="4">D14*3.28084</f>
         <v>1.64042E-12</v>
       </c>
-      <c r="E11" s="3">
-        <f t="shared" si="0"/>
+      <c r="E15" s="9">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="F11" s="3">
-        <f t="shared" si="0"/>
+      <c r="F15" s="9">
+        <f t="shared" si="4"/>
         <v>1.64042E-10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="14">
+        <v>5</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="15">
+        <f>D15*86400</f>
+        <v>1.41732288E-7</v>
+      </c>
+      <c r="E16" s="15">
+        <f t="shared" ref="E16:F16" si="5">E15*86400</f>
+        <v>0</v>
+      </c>
+      <c r="F16" s="15">
+        <f t="shared" si="5"/>
+        <v>1.41732288E-5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>